<commit_message>
Session 21 close: Notion portfolio page published + tracking files updated
Portfolio page live: https://rust-teal-362.notion.site/Muhammed-Ashnad-Finance-Portfolio-3cce8e1148b0800aa16feeb11a1e7bdc
Contains: 3 charts, full project copy, downloadable Zara_Co_FPA_Model_2025.xlsx.
DAILY_LOG, CHANGELOG, PENDING, PHASE2_MASTER_PLAN updated.
FP&A model build scripts added to repo (add_cogs_tab.py, add_opex_tab.py, etc.).
Project 1 now 95% — LinkedIn post is the only remaining step.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GDkSADdjhpopLb3RfxLaxD
</commit_message>
<xml_diff>
--- a/learning/phase2b_project1/08_fpa_model.xlsx
+++ b/learning/phase2b_project1/08_fpa_model.xlsx
@@ -8130,8 +8130,8 @@
     <row r="20" ht="50" customHeight="1" s="130">
       <c r="A20" s="129" t="inlineStr">
         <is>
-          <t>Paragraph 2 — OpEx &amp; EBITDA:
-EBITDA fell short by AED 91K (-10.1%) for the quarter, driven by two factors: a cumulative gross profit miss of AED 229K and an OpEx overspend of AED 70K (+3.4%). Marketing costs ran above plan in all three months, with March showing the largest deviation at AED 43K above budget. The combined effect compressed EBITDA margin by approximately 4.5 percentage points versus budget.</t>
+          <t>Paragraph 2 — OpEx &amp; Operating Profit:
+Operating Profit fell short by AED 141K (-10.1%) for the quarter, driven by two factors: a cumulative gross profit miss of AED 74K and an OpEx overspend of AED 70K (+3.4%). Marketing costs ran above plan in all three months, with March showing the largest deviation at AED 43K above budget. The combined effect compressed operating margin by 200 basis points (2.0pp) versus budget.</t>
         </is>
       </c>
     </row>

</xml_diff>